<commit_message>
case04 dei test di laboratorio
corretto il test04 dei referti di laboratorio, aggiornato data.json e checklist
</commit_message>
<xml_diff>
--- a/GATEWAY/S1#111INNOVATIONG/INNOVATIONGROUP/NOVALAB/8.4/accreditamento-checklist_V8.3.0.xlsx
+++ b/GATEWAY/S1#111INNOVATIONG/INNOVATIONGROUP/NOVALAB/8.4/accreditamento-checklist_V8.3.0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\FSE-Tools\allyouneed\LAB\GATEWAY\S1#111INNOVATIONG\INNOVATIONGROUP\NOVALAB\8.4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEBAF2CB-EF4E-4F8C-B228-B58252BDFD01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC974A83-2E31-494A-A533-BE2C7775942D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Istruzioni Compilazione" sheetId="1" r:id="rId1"/>
@@ -36,8 +36,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -2089,15 +2087,6 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 6" riportata nei documenti "casi di test TPI" e "CDA2_Tessera_Portatore_Impianto_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento. </t>
   </si>
   <si>
-    <t>2026-03-09T09:12:43Z</t>
-  </si>
-  <si>
-    <t>fcd7b0551b8a014f5544d3b7b0014cf7</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.150.4.4.cd42edb80cb67dc045b7c0a22882ce4eab8e08e2de5305813ce291a4deabe880.d67b9b2cc2^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>2026-03-09T14:47:42Z</t>
   </si>
   <si>
@@ -2288,6 +2277,15 @@
   </si>
   <si>
     <t>subject_application_version: 8.4</t>
+  </si>
+  <si>
+    <t>2026-03-24T14:49:53Z</t>
+  </si>
+  <si>
+    <t>0ef3e965d73d1016b38e82b3869307f2</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.150.4.4.cd42edb80cb67dc045b7c0a22882ce4eab8  e08e2de5305813ce291a4deabe880.78d70eb1e3^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -4406,7 +4404,7 @@
       </c>
       <c r="B2" s="57"/>
       <c r="C2" s="58" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="D2" s="57"/>
       <c r="F2" s="6"/>
@@ -4434,7 +4432,7 @@
       </c>
       <c r="B3" s="60"/>
       <c r="C3" s="65" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="D3" s="57"/>
       <c r="F3" s="6"/>
@@ -4460,7 +4458,7 @@
       <c r="A4" s="61"/>
       <c r="B4" s="62"/>
       <c r="C4" s="65" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
       <c r="D4" s="57"/>
       <c r="E4" s="4"/>
@@ -4487,7 +4485,7 @@
       <c r="A5" s="63"/>
       <c r="B5" s="64"/>
       <c r="C5" s="65" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="D5" s="57"/>
       <c r="F5" s="6"/>
@@ -4663,16 +4661,16 @@
         <v>46</v>
       </c>
       <c r="F10" s="34">
-        <v>46090</v>
+        <v>46105</v>
       </c>
       <c r="G10" s="34" t="s">
-        <v>546</v>
+        <v>610</v>
       </c>
       <c r="H10" s="34" t="s">
-        <v>547</v>
+        <v>611</v>
       </c>
       <c r="I10" s="35" t="s">
-        <v>548</v>
+        <v>612</v>
       </c>
       <c r="J10" s="36" t="s">
         <v>76</v>
@@ -4713,10 +4711,10 @@
         <v>46090</v>
       </c>
       <c r="G11" s="35" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="H11" s="35" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="I11" s="40"/>
       <c r="J11" s="36" t="s">
@@ -4731,7 +4729,7 @@
         <v>76</v>
       </c>
       <c r="O11" s="36" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="P11" s="36" t="s">
         <v>76</v>
@@ -4739,7 +4737,7 @@
       <c r="Q11" s="36"/>
       <c r="R11" s="36"/>
       <c r="S11" s="36" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="T11" s="36"/>
       <c r="U11" s="37"/>
@@ -5027,10 +5025,10 @@
         <v>46090</v>
       </c>
       <c r="G19" s="35" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
       <c r="H19" s="35" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="I19" s="40"/>
       <c r="J19" s="36" t="s">
@@ -5045,7 +5043,7 @@
         <v>76</v>
       </c>
       <c r="O19" s="36" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="P19" s="36" t="s">
         <v>76</v>
@@ -5053,7 +5051,7 @@
       <c r="Q19" s="36"/>
       <c r="R19" s="36"/>
       <c r="S19" s="36" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="T19" s="36"/>
       <c r="U19" s="37"/>
@@ -5341,7 +5339,7 @@
         <v>46090</v>
       </c>
       <c r="G27" s="35" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="H27" s="35"/>
       <c r="I27" s="40"/>
@@ -5357,7 +5355,7 @@
         <v>76</v>
       </c>
       <c r="O27" s="36" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="P27" s="36" t="s">
         <v>76</v>
@@ -5365,7 +5363,7 @@
       <c r="Q27" s="36"/>
       <c r="R27" s="36"/>
       <c r="S27" s="36" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="T27" s="36"/>
       <c r="U27" s="37" t="s">
@@ -5669,13 +5667,13 @@
         <v>46090</v>
       </c>
       <c r="G35" s="35" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="H35" s="35" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="I35" s="40" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="J35" s="36" t="s">
         <v>76</v>
@@ -5689,7 +5687,7 @@
         <v>76</v>
       </c>
       <c r="O35" s="36" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="P35" s="36" t="s">
         <v>76</v>
@@ -5697,7 +5695,7 @@
       <c r="Q35" s="36"/>
       <c r="R35" s="36"/>
       <c r="S35" s="36" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="T35" s="36"/>
       <c r="U35" s="37"/>
@@ -5726,13 +5724,13 @@
         <v>46091</v>
       </c>
       <c r="G36" s="35" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="H36" s="35" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="I36" s="40" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="J36" s="36" t="s">
         <v>76</v>
@@ -5746,7 +5744,7 @@
         <v>76</v>
       </c>
       <c r="O36" s="36" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="P36" s="36" t="s">
         <v>76</v>
@@ -5754,7 +5752,7 @@
       <c r="Q36" s="36"/>
       <c r="R36" s="36"/>
       <c r="S36" s="36" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="T36" s="36"/>
       <c r="U36" s="37"/>
@@ -5783,13 +5781,13 @@
         <v>46091</v>
       </c>
       <c r="G37" s="35" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="H37" s="35" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="I37" s="40" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="J37" s="36" t="s">
         <v>76</v>
@@ -5803,7 +5801,7 @@
         <v>76</v>
       </c>
       <c r="O37" s="36" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="P37" s="36" t="s">
         <v>76</v>
@@ -5811,7 +5809,7 @@
       <c r="Q37" s="36"/>
       <c r="R37" s="36"/>
       <c r="S37" s="36" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="T37" s="36"/>
       <c r="U37" s="37"/>
@@ -5840,13 +5838,13 @@
         <v>46091</v>
       </c>
       <c r="G38" s="35" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="H38" s="35" t="s">
-        <v>573</v>
+        <v>570</v>
       </c>
       <c r="I38" s="40" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="J38" s="36" t="s">
         <v>76</v>
@@ -5860,7 +5858,7 @@
         <v>76</v>
       </c>
       <c r="O38" s="36" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="P38" s="36" t="s">
         <v>76</v>
@@ -5868,7 +5866,7 @@
       <c r="Q38" s="36"/>
       <c r="R38" s="36"/>
       <c r="S38" s="36" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="T38" s="36"/>
       <c r="U38" s="37"/>
@@ -5897,13 +5895,13 @@
         <v>46091</v>
       </c>
       <c r="G39" s="35" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
       <c r="H39" s="35" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="I39" s="40" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="J39" s="36" t="s">
         <v>76</v>
@@ -5917,7 +5915,7 @@
         <v>76</v>
       </c>
       <c r="O39" s="36" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
       <c r="P39" s="36" t="s">
         <v>76</v>
@@ -5925,7 +5923,7 @@
       <c r="Q39" s="36"/>
       <c r="R39" s="36"/>
       <c r="S39" s="36" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="T39" s="36"/>
       <c r="U39" s="37"/>
@@ -5954,13 +5952,13 @@
         <v>46091</v>
       </c>
       <c r="G40" s="35" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="H40" s="35" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="I40" s="40" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="J40" s="36" t="s">
         <v>76</v>
@@ -5974,7 +5972,7 @@
         <v>76</v>
       </c>
       <c r="O40" s="36" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="P40" s="36" t="s">
         <v>76</v>
@@ -5982,7 +5980,7 @@
       <c r="Q40" s="36"/>
       <c r="R40" s="36"/>
       <c r="S40" s="36" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="T40" s="36"/>
       <c r="U40" s="37"/>
@@ -6011,13 +6009,13 @@
         <v>46092</v>
       </c>
       <c r="G41" s="35" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
       <c r="H41" s="35" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
       <c r="I41" s="40" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="J41" s="36" t="s">
         <v>76</v>
@@ -6031,7 +6029,7 @@
         <v>76</v>
       </c>
       <c r="O41" s="36" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
       <c r="P41" s="36" t="s">
         <v>76</v>
@@ -6039,7 +6037,7 @@
       <c r="Q41" s="36"/>
       <c r="R41" s="36"/>
       <c r="S41" s="36" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="T41" s="36"/>
       <c r="U41" s="37"/>
@@ -6068,13 +6066,13 @@
         <v>46094</v>
       </c>
       <c r="G42" s="35" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
       <c r="H42" s="35" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
       <c r="I42" s="40" t="s">
-        <v>590</v>
+        <v>587</v>
       </c>
       <c r="J42" s="36" t="s">
         <v>76</v>
@@ -6088,7 +6086,7 @@
         <v>76</v>
       </c>
       <c r="O42" s="36" t="s">
-        <v>591</v>
+        <v>588</v>
       </c>
       <c r="P42" s="36" t="s">
         <v>76</v>
@@ -6096,7 +6094,7 @@
       <c r="Q42" s="36"/>
       <c r="R42" s="36"/>
       <c r="S42" s="36" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="T42" s="36"/>
       <c r="U42" s="37"/>
@@ -9936,13 +9934,13 @@
         <v>46094</v>
       </c>
       <c r="G146" s="35" t="s">
-        <v>592</v>
+        <v>589</v>
       </c>
       <c r="H146" s="35" t="s">
-        <v>593</v>
+        <v>590</v>
       </c>
       <c r="I146" s="40" t="s">
-        <v>594</v>
+        <v>591</v>
       </c>
       <c r="J146" s="36" t="s">
         <v>76</v>
@@ -9985,13 +9983,13 @@
         <v>46094</v>
       </c>
       <c r="G147" s="35" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
       <c r="H147" s="35" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
       <c r="I147" s="40" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
       <c r="J147" s="36" t="s">
         <v>76</v>
@@ -10776,13 +10774,13 @@
         <v>46094</v>
       </c>
       <c r="G168" s="35" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="H168" s="35" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="I168" s="40" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="J168" s="36" t="s">
         <v>76</v>
@@ -11269,13 +11267,13 @@
         <v>46094</v>
       </c>
       <c r="G181" s="33" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="H181" s="33" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="I181" s="36" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="J181" s="36" t="s">
         <v>76</v>
@@ -11289,7 +11287,7 @@
         <v>76</v>
       </c>
       <c r="O181" s="36" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
       <c r="P181" s="36" t="s">
         <v>76</v>
@@ -11297,7 +11295,7 @@
       <c r="Q181" s="36"/>
       <c r="R181" s="36"/>
       <c r="S181" s="36" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="T181" s="36"/>
       <c r="U181" s="33"/>
@@ -11548,13 +11546,13 @@
         <v>46094</v>
       </c>
       <c r="G188" s="35" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="H188" s="35" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="I188" s="40" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
       <c r="J188" s="36" t="s">
         <v>76</v>
@@ -11568,7 +11566,7 @@
         <v>76</v>
       </c>
       <c r="O188" s="36" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="P188" s="36" t="s">
         <v>76</v>
@@ -11576,7 +11574,7 @@
       <c r="Q188" s="36"/>
       <c r="R188" s="36"/>
       <c r="S188" s="36" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="T188" s="36"/>
       <c r="U188" s="37"/>
@@ -19003,15 +19001,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A92AB09DCDF6014AA0D6826BF29E2C8E" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="58b13f75919cba2dcad85f84b1d5db00">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1e76d14e-d0ce-457c-8343-9b55836d9ead" xmlns:ns3="a56712a3-8dfd-4688-917a-22f0cf513b89" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a3b16ea44285e6579c272a3325f660d0" ns2:_="" ns3:_="">
     <xsd:import namespace="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
@@ -19275,6 +19264,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -19288,14 +19286,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C578C2C-7E0B-429D-96B0-25A2E02D9084}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19310,6 +19300,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
correzione case 4 Lab
WII_UNKNOWN_TRANSACTION
</commit_message>
<xml_diff>
--- a/GATEWAY/S1#111INNOVATIONG/INNOVATIONGROUP/NOVALAB/8.4/accreditamento-checklist_V8.3.0.xlsx
+++ b/GATEWAY/S1#111INNOVATIONG/INNOVATIONGROUP/NOVALAB/8.4/accreditamento-checklist_V8.3.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\FSE-Tools\allyouneed\LAB\GATEWAY\S1#111INNOVATIONG\INNOVATIONGROUP\NOVALAB\8.4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC974A83-2E31-494A-A533-BE2C7775942D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98728730-51AA-493D-A1F2-530694C4FA79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2285,7 +2285,7 @@
     <t>0ef3e965d73d1016b38e82b3869307f2</t>
   </si>
   <si>
-    <t>2.16.840.1.113883.2.9.2.150.4.4.cd42edb80cb67dc045b7c0a22882ce4eab8  e08e2de5305813ce291a4deabe880.78d70eb1e3^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>2.16.840.1.113883.2.9.2.150.4.4.cd42edb80cb67dc045b7c0a22882ce4eab8e08e2de5305813ce291a4deabe880.78d70eb1e3^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -19001,6 +19001,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A92AB09DCDF6014AA0D6826BF29E2C8E" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="58b13f75919cba2dcad85f84b1d5db00">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1e76d14e-d0ce-457c-8343-9b55836d9ead" xmlns:ns3="a56712a3-8dfd-4688-917a-22f0cf513b89" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a3b16ea44285e6579c272a3325f660d0" ns2:_="" ns3:_="">
     <xsd:import namespace="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
@@ -19264,15 +19273,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -19286,6 +19286,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C578C2C-7E0B-429D-96B0-25A2E02D9084}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19300,14 +19308,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>